<commit_message>
rename node_state_cap to capacity for storages example data.
</commit_message>
<xml_diff>
--- a/example_data/storages/storages-input.xlsx
+++ b/example_data/storages/storages-input.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="42">
   <si>
     <t xml:space="preserve">block_identifier</t>
   </si>
@@ -32,61 +32,64 @@
     <t xml:space="preserve">alternative_name</t>
   </si>
   <si>
+    <t xml:space="preserve">capacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_charging</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_discharging</t>
+  </si>
+  <si>
+    <t xml:space="preserve">demand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unit_investment_cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">storage_investment_cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">candidate_units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">candidate_storages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">storage_investment_variable_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">emissionnode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">investment_emission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">emission_cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explanation of the data columns in Sheet1:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">column</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name of the city block where the production unit lies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“heat” for heating heat storages, “elec” for electricity storages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternative which the given values are for</t>
+  </si>
+  <si>
     <t xml:space="preserve">node_state_cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_charging</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_discharging</t>
-  </si>
-  <si>
-    <t xml:space="preserve">demand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unit_investment_cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">storage_investment_cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">candidate_units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">candidate_storages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">storage_investment_variable_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">emissionnode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">investment_emission</t>
-  </si>
-  <si>
-    <t xml:space="preserve">emission_cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explanation of the data columns in Sheet1:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">column</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">name of the city block where the production unit lies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">“heat” for heating heat storages, “elec” for electricity storages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alternative which the given values are for</t>
   </si>
   <si>
     <t xml:space="preserve">Capacity of one storage unit</t>
@@ -533,7 +536,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" objects="true" scenarios="true"/>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="L2:L1001" type="list">
       <formula1>"storage_investment_variable_type_continuous,storage_investment_variable_type_integer"</formula1>
@@ -608,13 +610,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -622,10 +624,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -633,10 +635,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>26</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -644,10 +646,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -655,10 +657,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -666,10 +668,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>30</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -677,7 +679,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C13" s="8"/>
     </row>
@@ -686,7 +688,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C14" s="8"/>
     </row>
@@ -702,7 +704,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C16" s="8"/>
     </row>
@@ -711,10 +713,10 @@
         <v>13</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -722,23 +724,23 @@
         <v>14</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>